<commit_message>
Adicionar script para colorir células e gerar legenda no Excel
</commit_message>
<xml_diff>
--- a/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
+++ b/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Página1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGENDA" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15,7 +16,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -41,8 +42,19 @@
       <name val="Arial"/>
       <color theme="1"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="43">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +77,196 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
         <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F78888"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DA88F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BE6FF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F756D5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0089F762"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F77A62"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005691F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B6F788"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7A27B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CDF756"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0062F7B1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F76FC5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0088F77B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F76291"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F77BF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0088E5F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0062C8F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7A256"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00888DF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0056F7DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E762F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7EF62"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0056F75F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F77B8F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7C56F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007BBCF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007BF7D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006FF78B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0088F7B1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F788BC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009C7BF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007262F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006FF7F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF77B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BEF76F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7DF88"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009A56F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006F8BF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -123,7 +325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -153,6 +355,159 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="38" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="39" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="40" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="41" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="42" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,67 +886,67 @@
       <c r="B2" s="3" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="20" t="inlineStr">
         <is>
           <t>DRIELLI- INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="21" t="inlineStr">
         <is>
           <t>ANDREA- MATEMÁTICA APL</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="N2" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="25" t="inlineStr">
         <is>
           <t>GERALDO- EMPREEN</t>
         </is>
@@ -602,67 +957,67 @@
       <c r="B3" s="3" t="n">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
         <is>
           <t>DRIELLI- INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="21" t="inlineStr">
         <is>
           <t>ANDREA- MATEMÁTICA APL</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="25" t="inlineStr">
         <is>
           <t>GERALDO- EMPREEN</t>
         </is>
@@ -673,67 +1028,67 @@
       <c r="B4" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="26" t="inlineStr">
         <is>
           <t>THOMAZ- HIST</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="21" t="inlineStr">
         <is>
           <t>ANDREA- MATEMÁTICA APL</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="20" t="inlineStr">
         <is>
           <t>DRIELLI- INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="O4" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
@@ -744,67 +1099,67 @@
       <c r="B5" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>ANDREA- MATEMÁTICA APL</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="20" t="inlineStr">
         <is>
           <t>DRIELLI- INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
@@ -836,67 +1191,67 @@
       <c r="B7" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="20" t="inlineStr">
         <is>
           <t>DRIELLI- CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="21" t="inlineStr">
         <is>
           <t>ANDREA- GESTÃO DE OPER.</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="N7" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="O7" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
@@ -907,67 +1262,67 @@
       <c r="B8" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="20" t="inlineStr">
         <is>
           <t>DRIELLI- CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="21" t="inlineStr">
         <is>
           <t>ANDREA- GESTÃO DE OPER.</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="N8" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="O8" s="4" t="inlineStr">
+      <c r="O8" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
@@ -982,67 +1337,67 @@
       <c r="B9" s="3" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE LP</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="31" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K9" s="32" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="N9" s="33" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="O9" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
@@ -1053,67 +1408,67 @@
       <c r="B10" s="3" t="n">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE LP</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="31" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K10" s="32" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="N10" s="33" t="inlineStr">
         <is>
           <t>SAMIA- AP SOC</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="O10" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
@@ -1124,67 +1479,67 @@
       <c r="B11" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>SILVANA- RED</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="32" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K11" s="31" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="N11" s="33" t="inlineStr">
         <is>
           <t>SAMIA- AP SOC</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
+      <c r="O11" s="18" t="inlineStr">
         <is>
           <t>ALINE- SOC</t>
         </is>
@@ -1195,67 +1550,67 @@
       <c r="B12" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>SILVANA- RED</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="32" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K12" s="31" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" s="33" t="inlineStr">
         <is>
           <t>SAMIA- ARTE E MÍDIA</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N12" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
+      <c r="O12" s="18" t="inlineStr">
         <is>
           <t>ALINE- SOC</t>
         </is>
@@ -1287,67 +1642,67 @@
       <c r="B14" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="33" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I14" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="34" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M14" s="35" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="N14" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="O14" s="4" t="inlineStr">
+      <c r="O14" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE PORT</t>
         </is>
@@ -1358,67 +1713,67 @@
       <c r="B15" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
         <is>
           <t>THOMAZ- HIST</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I15" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J15" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K15" s="34" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L15" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="35" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="N15" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
+      <c r="O15" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE PORT</t>
         </is>
@@ -1433,67 +1788,67 @@
       <c r="B16" s="3" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I16" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K16" s="34" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L16" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M16" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="N16" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="O16" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
@@ -1504,67 +1859,67 @@
       <c r="B17" s="3" t="n">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I17" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K17" s="34" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L17" s="33" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M17" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="N17" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="O17" s="4" t="inlineStr">
+      <c r="O17" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
@@ -1575,67 +1930,67 @@
       <c r="B18" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I18" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" s="33" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="K18" s="37" t="inlineStr">
         <is>
           <t>BENEDITA- GEO</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L18" s="22" t="inlineStr">
         <is>
           <t>DAVI- EFIN</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="M18" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="N18" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="O18" s="4" t="inlineStr">
+      <c r="O18" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
@@ -1646,67 +2001,67 @@
       <c r="B19" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K19" s="37" t="inlineStr">
         <is>
           <t>BENEDITA- GEO</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L19" s="22" t="inlineStr">
         <is>
           <t>DAVI- EFIN</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M19" s="39" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="N19" s="33" t="inlineStr">
         <is>
           <t>SAMIA- AP FIL</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr">
+      <c r="O19" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
@@ -1738,67 +2093,67 @@
       <c r="B21" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>SILVANA- RED</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J21" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="L21" s="18" t="inlineStr">
         <is>
           <t>ALINE- ORATÓRIA</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="M21" s="39" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="N21" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr">
+      <c r="O21" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
@@ -1809,67 +2164,67 @@
       <c r="B22" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>THOMAZ- HIST</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="27" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>SILVANA- RED</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I22" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L22" s="18" t="inlineStr">
         <is>
           <t>ALINE- ORATÓRIA</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M22" s="39" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="N22" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="O22" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
@@ -1884,67 +2239,67 @@
       <c r="B23" s="3" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="19" t="inlineStr">
         <is>
           <t>MARINA- PORT</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="24" t="inlineStr">
         <is>
           <t>SILVIA- EFIN</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J23" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="K23" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="L23" s="33" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="M23" s="40" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="N23" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
+      <c r="O23" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- AP QUIM</t>
         </is>
@@ -1955,67 +2310,67 @@
       <c r="B24" s="3" t="n">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>MARINA- PORT</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" s="24" t="inlineStr">
         <is>
           <t>SILVIA- EFIN</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" s="33" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="K24" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="M24" s="40" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="N24" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="O24" s="4" t="inlineStr">
+      <c r="O24" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
@@ -2026,67 +2381,67 @@
       <c r="B25" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="33" t="inlineStr">
         <is>
           <t>SAMIA- ARTE</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="J25" s="37" t="inlineStr">
         <is>
           <t>BENEDITA- GEO</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="K25" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="M25" s="41" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="N25" s="42" t="inlineStr">
         <is>
           <t>SIMARA- OE LP</t>
         </is>
       </c>
-      <c r="O25" s="4" t="inlineStr">
+      <c r="O25" s="24" t="inlineStr">
         <is>
           <t>SILVIA- OE MAT</t>
         </is>
@@ -2097,67 +2452,67 @@
       <c r="B26" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="33" t="inlineStr">
         <is>
           <t>SAMIA- ARTE</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H26" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J26" s="37" t="inlineStr">
         <is>
           <t>BENEDITA- GEO</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="K26" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L26" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="M26" s="43" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
       </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="N26" s="42" t="inlineStr">
         <is>
           <t>SIMARA- OE LP</t>
         </is>
       </c>
-      <c r="O26" s="4" t="inlineStr">
+      <c r="O26" s="24" t="inlineStr">
         <is>
           <t>SILVIA- OE MAT</t>
         </is>
@@ -2189,67 +2544,67 @@
       <c r="B28" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="44" t="inlineStr">
         <is>
           <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H28" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J28" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="K28" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L28" s="45" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="M28" s="46" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="N28" s="47" t="inlineStr">
         <is>
           <t>DINO- AP GEO</t>
         </is>
       </c>
-      <c r="O28" s="4" t="inlineStr">
+      <c r="O28" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
@@ -2260,67 +2615,67 @@
       <c r="B29" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F29" s="44" t="inlineStr">
         <is>
           <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G29" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H29" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I29" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J29" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="K29" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L29" s="45" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="M29" s="46" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="N29" s="47" t="inlineStr">
         <is>
           <t>DINO- AP GEO</t>
         </is>
       </c>
-      <c r="O29" s="4" t="inlineStr">
+      <c r="O29" s="48" t="inlineStr">
         <is>
           <t>BORTOLOTI- PROG</t>
         </is>
@@ -2335,67 +2690,67 @@
       <c r="B30" s="3" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="33" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="47" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H30" s="45" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J30" s="49" t="inlineStr">
         <is>
           <t>RAFAEL- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="K30" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="M30" s="46" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="N30" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="O30" s="4" t="inlineStr">
+      <c r="O30" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
@@ -2406,67 +2761,67 @@
       <c r="B31" s="3" t="n">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="19" t="inlineStr">
         <is>
           <t>MARINA- PORT</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="47" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="45" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I31" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J31" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="K31" s="33" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" s="38" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="M31" s="43" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="N31" s="24" t="inlineStr">
         <is>
           <t>SILVIA- OE MAT</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr">
+      <c r="O31" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- AP QUIM</t>
         </is>
@@ -2477,67 +2832,67 @@
       <c r="B32" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="19" t="inlineStr">
         <is>
           <t>MARINA- PORT</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="47" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="25" t="inlineStr">
         <is>
           <t>GERALDO- OE MAT</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="45" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H32" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="K32" s="33" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L32" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="M32" s="43" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
       </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="N32" s="17" t="inlineStr">
         <is>
           <t>EUNICE- ATUALID</t>
         </is>
       </c>
-      <c r="O32" s="4" t="inlineStr">
+      <c r="O32" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
@@ -2548,67 +2903,67 @@
       <c r="B33" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="47" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="25" t="inlineStr">
         <is>
           <t>GERALDO- OE MAT</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="45" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H33" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I33" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="J33" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="K33" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L33" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="M33" s="50" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
       </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="N33" s="24" t="inlineStr">
         <is>
           <t>SILVIA- OE MAT</t>
         </is>
       </c>
-      <c r="O33" s="4" t="inlineStr">
+      <c r="O33" s="33" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
@@ -2640,67 +2995,67 @@
       <c r="B35" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="47" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G35" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H35" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I35" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J35" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="K35" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L35" s="45" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="M35" s="50" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
       </c>
-      <c r="N35" s="4" t="inlineStr">
+      <c r="N35" s="33" t="inlineStr">
         <is>
           <t>SAMIA- AP FILO</t>
         </is>
       </c>
-      <c r="O35" s="4" t="inlineStr">
+      <c r="O35" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
@@ -2711,67 +3066,67 @@
       <c r="B36" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="47" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="29" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H36" s="36" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I36" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="J36" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="K36" s="13" t="inlineStr">
         <is>
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="L36" s="45" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="M36" s="50" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
       </c>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="N36" s="17" t="inlineStr">
         <is>
           <t>EUNICE- ATUALID</t>
         </is>
       </c>
-      <c r="O36" s="4" t="inlineStr">
+      <c r="O36" s="48" t="inlineStr">
         <is>
           <t>BORTOLOTI- PROG</t>
         </is>
@@ -3751,4 +4106,338 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="9" min="1" max="1"/>
+    <col width="14" customWidth="1" style="9" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="51" t="inlineStr">
+        <is>
+          <t>PROFESSOR / DISCIPLINA</t>
+        </is>
+      </c>
+      <c r="B1" s="51" t="inlineStr">
+        <is>
+          <t>COR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ALEXANDRE</t>
+        </is>
+      </c>
+      <c r="B2" s="52" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ALINE</t>
+        </is>
+      </c>
+      <c r="B3" s="53" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ANDREA</t>
+        </is>
+      </c>
+      <c r="B4" s="54" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BAQUETE</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BENEDITA</t>
+        </is>
+      </c>
+      <c r="B6" s="56" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BORTOLOTI</t>
+        </is>
+      </c>
+      <c r="B7" s="57" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CARREIRA E COMP</t>
+        </is>
+      </c>
+      <c r="B8" s="58" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>COMUNICAÇÃO</t>
+        </is>
+      </c>
+      <c r="B9" s="59" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DAVI</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DINO</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DRIELLI</t>
+        </is>
+      </c>
+      <c r="B12" s="62" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EUNICE</t>
+        </is>
+      </c>
+      <c r="B13" s="63" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GERALDO</t>
+        </is>
+      </c>
+      <c r="B14" s="64" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GEST. FINANCEIRA</t>
+        </is>
+      </c>
+      <c r="B15" s="65" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GESTÃO DE OPERAÇÕES</t>
+        </is>
+      </c>
+      <c r="B16" s="66" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GESTÃO FINANCEIRA</t>
+        </is>
+      </c>
+      <c r="B17" s="67" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GISELE</t>
+        </is>
+      </c>
+      <c r="B18" s="68" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>INOVAÇÃO E DES</t>
+        </is>
+      </c>
+      <c r="B19" s="69" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>INTRODUÇÃO ADM</t>
+        </is>
+      </c>
+      <c r="B20" s="70" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LILIANE</t>
+        </is>
+      </c>
+      <c r="B21" s="71" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>M.EDUARDA</t>
+        </is>
+      </c>
+      <c r="B22" s="72" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>MARCIA</t>
+        </is>
+      </c>
+      <c r="B23" s="73" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MARIANA</t>
+        </is>
+      </c>
+      <c r="B24" s="74" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MARINA</t>
+        </is>
+      </c>
+      <c r="B25" s="75" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MARKETING</t>
+        </is>
+      </c>
+      <c r="B26" s="76" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MAT APLICADA</t>
+        </is>
+      </c>
+      <c r="B27" s="77" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PAPANONI</t>
+        </is>
+      </c>
+      <c r="B28" s="78" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PROJETO MULTI</t>
+        </is>
+      </c>
+      <c r="B29" s="79" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>RAFAEL</t>
+        </is>
+      </c>
+      <c r="B30" s="80" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ROBERTA</t>
+        </is>
+      </c>
+      <c r="B31" s="81" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ROMARIO</t>
+        </is>
+      </c>
+      <c r="B32" s="82" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SAMIA</t>
+        </is>
+      </c>
+      <c r="B33" s="83" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SELMA</t>
+        </is>
+      </c>
+      <c r="B34" s="84" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SILVANA</t>
+        </is>
+      </c>
+      <c r="B35" s="85" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SILVIA</t>
+        </is>
+      </c>
+      <c r="B36" s="86" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SIMARA</t>
+        </is>
+      </c>
+      <c r="B37" s="87" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>THOMAZ</t>
+        </is>
+      </c>
+      <c r="B38" s="88" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>VINICIUS</t>
+        </is>
+      </c>
+      <c r="B39" s="89" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adicionar scripts de otimização para agendamento de professores e resolução de conflitos
</commit_message>
<xml_diff>
--- a/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
+++ b/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
@@ -903,7 +903,7 @@
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
+          <t>SILVANA- RED</t>
         </is>
       </c>
       <c r="G2" s="17" t="inlineStr">
@@ -933,12 +933,12 @@
       </c>
       <c r="L2" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>DAVI- EFIN</t>
         </is>
       </c>
       <c r="M2" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="N2" s="24" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="O2" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
@@ -979,47 +979,47 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>DRIELLI- INTRODUÇÃO ADM</t>
+        </is>
+      </c>
+      <c r="K3" s="21" t="inlineStr">
+        <is>
+          <t>ANDREA- MATEMÁTICA APL</t>
+        </is>
+      </c>
+      <c r="L3" s="23" t="inlineStr">
+        <is>
+          <t>DAVI- EFIN</t>
+        </is>
+      </c>
+      <c r="M3" s="22" t="inlineStr">
+        <is>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="N3" s="24" t="inlineStr">
+        <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="I3" s="19" t="inlineStr">
-        <is>
-          <t>MARINA- REDAÇÃO</t>
-        </is>
-      </c>
-      <c r="J3" s="20" t="inlineStr">
-        <is>
-          <t>DRIELLI- INTRODUÇÃO ADM</t>
-        </is>
-      </c>
-      <c r="K3" s="21" t="inlineStr">
-        <is>
-          <t>ANDREA- MATEMÁTICA APL</t>
-        </is>
-      </c>
-      <c r="L3" s="23" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="M3" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="N3" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
       <c r="O3" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C4" s="26" t="inlineStr">
         <is>
-          <t>THOMAZ- HIST</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="D4" s="27" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="I4" s="18" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="J4" s="21" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O4" s="28" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="D5" s="27" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="N5" s="22" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="O5" s="28" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="K7" s="18" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="L7" s="19" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="N7" s="28" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="O7" s="22" t="inlineStr">
@@ -1279,47 +1279,47 @@
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>DRIELLI- CARREIRA E COMP</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="L8" s="19" t="inlineStr">
+        <is>
+          <t>MARINA- REDAÇÃO</t>
+        </is>
+      </c>
+      <c r="M8" s="21" t="inlineStr">
+        <is>
+          <t>ANDREA- GESTÃO DE OPER.</t>
+        </is>
+      </c>
+      <c r="N8" s="28" t="inlineStr">
+        <is>
           <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="J8" s="20" t="inlineStr">
-        <is>
-          <t>DRIELLI- CARREIRA E COMP</t>
-        </is>
-      </c>
-      <c r="K8" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="L8" s="19" t="inlineStr">
-        <is>
-          <t>MARINA- REDAÇÃO</t>
-        </is>
-      </c>
-      <c r="M8" s="21" t="inlineStr">
-        <is>
-          <t>ANDREA- GESTÃO DE OPER.</t>
-        </is>
-      </c>
-      <c r="N8" s="28" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O8" s="22" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -1354,44 +1354,44 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
+          <t>PAPANONI- ED. FINAN</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="G9" s="29" t="inlineStr">
-        <is>
-          <t>MARCIA- ARTE</t>
-        </is>
-      </c>
       <c r="H9" s="22" t="inlineStr">
         <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="J9" s="31" t="inlineStr">
+        <is>
+          <t>MAT APLICADA</t>
+        </is>
+      </c>
+      <c r="K9" s="32" t="inlineStr">
+        <is>
+          <t>INTRODUÇÃO ADM</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="I9" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="J9" s="31" t="inlineStr">
-        <is>
-          <t>MAT APLICADA</t>
-        </is>
-      </c>
-      <c r="K9" s="32" t="inlineStr">
-        <is>
-          <t>INTRODUÇÃO ADM</t>
-        </is>
-      </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="M9" s="28" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
       <c r="N9" s="33" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -1425,17 +1425,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="G10" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="H10" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="O10" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>DAVI- MAT</t>
         </is>
       </c>
       <c r="E11" s="30" t="inlineStr">
@@ -1501,17 +1501,17 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="H11" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="I11" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- EFIN</t>
         </is>
       </c>
       <c r="J11" s="32" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="L11" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="M11" s="17" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>ALINE- SOC</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="H12" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="I12" s="24" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="N12" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="O12" s="18" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="H14" s="24" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="I14" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="J14" s="34" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="O14" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="H15" s="24" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="I15" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J15" s="25" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="O15" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
     </row>
@@ -1805,52 +1805,52 @@
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="K16" s="34" t="inlineStr">
+        <is>
+          <t>CARREIRA E COMP</t>
+        </is>
+      </c>
+      <c r="L16" s="36" t="inlineStr">
+        <is>
+          <t>ALINE- ORATÓRIA</t>
+        </is>
+      </c>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>GERALDO- MAT</t>
+        </is>
+      </c>
+      <c r="N16" s="28" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
+        </is>
+      </c>
+      <c r="O16" s="23" t="inlineStr">
+        <is>
           <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="G16" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- FILOSOFIA</t>
-        </is>
-      </c>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="J16" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="K16" s="34" t="inlineStr">
-        <is>
-          <t>CARREIRA E COMP</t>
-        </is>
-      </c>
-      <c r="L16" s="36" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="M16" s="25" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
-        </is>
-      </c>
-      <c r="N16" s="28" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
-      <c r="O16" s="23" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1871,57 +1871,57 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
+          <t>ROMARIO- ED FÍSICA</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="F17" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="G17" s="22" t="inlineStr">
+      <c r="I17" s="36" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="K17" s="34" t="inlineStr">
+        <is>
+          <t>CARREIRA E COMP</t>
+        </is>
+      </c>
+      <c r="L17" s="33" t="inlineStr">
+        <is>
+          <t>SAMIA- SOC</t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>GERALDO- MAT</t>
+        </is>
+      </c>
+      <c r="N17" s="23" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- FILOSOFIA</t>
-        </is>
-      </c>
-      <c r="I17" s="36" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="J17" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="K17" s="34" t="inlineStr">
-        <is>
-          <t>CARREIRA E COMP</t>
-        </is>
-      </c>
-      <c r="L17" s="33" t="inlineStr">
-        <is>
-          <t>SAMIA- SOC</t>
-        </is>
-      </c>
-      <c r="M17" s="25" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
-        </is>
-      </c>
-      <c r="N17" s="23" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
       <c r="O17" s="28" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -1947,39 +1947,39 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- RED</t>
+        </is>
+      </c>
+      <c r="H18" s="24" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="I18" s="36" t="inlineStr">
+        <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="J18" s="33" t="inlineStr">
+        <is>
+          <t>SAMIA- SOC</t>
+        </is>
+      </c>
+      <c r="K18" s="37" t="inlineStr">
+        <is>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="L18" s="22" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="H18" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I18" s="36" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="J18" s="33" t="inlineStr">
-        <is>
-          <t>SAMIA- SOC</t>
-        </is>
-      </c>
-      <c r="K18" s="37" t="inlineStr">
-        <is>
-          <t>BENEDITA- GEO</t>
-        </is>
-      </c>
-      <c r="L18" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- EFIN</t>
-        </is>
-      </c>
       <c r="M18" s="28" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="N18" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>EUNICE- ATUALID</t>
         </is>
       </c>
       <c r="O18" s="13" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
@@ -2043,12 +2043,12 @@
       </c>
       <c r="K19" s="37" t="inlineStr">
         <is>
-          <t>BENEDITA- GEO</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="L19" s="22" t="inlineStr">
         <is>
-          <t>DAVI- EFIN</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="M19" s="39" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>GERALDO- OE MAT</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -2115,34 +2115,34 @@
       </c>
       <c r="G21" s="36" t="inlineStr">
         <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="I21" s="38" t="inlineStr">
+        <is>
+          <t>MARIANA- GEO</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="inlineStr">
+        <is>
+          <t>RAFAEL- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="L21" s="18" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="I21" s="38" t="inlineStr">
-        <is>
-          <t>MARIANA- GEO</t>
-        </is>
-      </c>
-      <c r="J21" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="L21" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- ORATÓRIA</t>
-        </is>
-      </c>
       <c r="M21" s="39" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
@@ -2150,12 +2150,12 @@
       </c>
       <c r="N21" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O21" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
     </row>
@@ -2176,17 +2176,17 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>GERALDO- OE MAT</t>
         </is>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="G22" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="J22" s="18" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -2221,12 +2221,12 @@
       </c>
       <c r="N22" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
     </row>
@@ -2261,22 +2261,22 @@
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- EFIN</t>
-        </is>
-      </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="K23" s="25" t="inlineStr">
@@ -2296,12 +2296,12 @@
       </c>
       <c r="N23" s="28" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>SIMARA- OE LP</t>
         </is>
       </c>
       <c r="O23" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- AP QUIM</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -2312,12 +2312,12 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>DAVI- MAT</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I24" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- EFIN</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="J24" s="33" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="L24" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="M24" s="40" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="N24" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>EUNICE- ATUALID</t>
         </is>
       </c>
       <c r="O24" s="28" t="inlineStr">
@@ -2383,14 +2383,14 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
+          <t>DAVI- MAT</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
           <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- MAT</t>
-        </is>
-      </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="I25" s="16" t="inlineStr">
@@ -2418,14 +2418,14 @@
       </c>
       <c r="J25" s="37" t="inlineStr">
         <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="K25" s="36" t="inlineStr">
+        <is>
           <t>BENEDITA- GEO</t>
         </is>
       </c>
-      <c r="K25" s="36" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
       <c r="L25" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
@@ -2438,12 +2438,12 @@
       </c>
       <c r="N25" s="42" t="inlineStr">
         <is>
-          <t>SIMARA- OE LP</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="D26" s="22" t="inlineStr">
@@ -2479,29 +2479,29 @@
       </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="J26" s="37" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="K26" s="36" t="inlineStr">
+        <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr">
+        <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="I26" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="J26" s="37" t="inlineStr">
-        <is>
-          <t>BENEDITA- GEO</t>
-        </is>
-      </c>
-      <c r="K26" s="36" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="L26" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
       <c r="M26" s="43" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="F28" s="44" t="inlineStr">
         <is>
-          <t>PAPANONI- ED. FINAN</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
@@ -2576,12 +2576,12 @@
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="J28" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K28" s="16" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="F29" s="44" t="inlineStr">
         <is>
-          <t>PAPANONI- ED. FINAN</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
@@ -2647,12 +2647,12 @@
       </c>
       <c r="I29" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="J29" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="O29" s="48" t="inlineStr">
         <is>
-          <t>BORTOLOTI- PROG</t>
+          <t>ALINE- SOC</t>
         </is>
       </c>
     </row>
@@ -2722,12 +2722,12 @@
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>SILVIA- EFIN</t>
         </is>
       </c>
       <c r="J30" s="49" t="inlineStr">
         <is>
-          <t>RAFAEL- ED. FÍSICA</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="K30" s="16" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="F31" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="G31" s="13" t="inlineStr">
@@ -2793,37 +2793,37 @@
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="K31" s="33" t="inlineStr">
+        <is>
+          <t>SAMIA- SOC</t>
+        </is>
+      </c>
+      <c r="L31" s="38" t="inlineStr">
+        <is>
+          <t>MARIANA- GEO</t>
+        </is>
+      </c>
+      <c r="M31" s="43" t="inlineStr">
+        <is>
+          <t>PROJETO MULTI</t>
+        </is>
+      </c>
+      <c r="N31" s="24" t="inlineStr">
+        <is>
+          <t>GERALDO- MAT</t>
+        </is>
+      </c>
+      <c r="O31" s="36" t="inlineStr">
+        <is>
           <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="J31" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="K31" s="33" t="inlineStr">
-        <is>
-          <t>SAMIA- SOC</t>
-        </is>
-      </c>
-      <c r="L31" s="38" t="inlineStr">
-        <is>
-          <t>MARIANA- GEO</t>
-        </is>
-      </c>
-      <c r="M31" s="43" t="inlineStr">
-        <is>
-          <t>PROJETO MULTI</t>
-        </is>
-      </c>
-      <c r="N31" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- OE MAT</t>
-        </is>
-      </c>
-      <c r="O31" s="36" t="inlineStr">
-        <is>
-          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D32" s="47" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="E32" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- OE MAT</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="F32" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="G32" s="45" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="H32" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="I32" s="22" t="inlineStr">
@@ -2889,12 +2889,12 @@
       </c>
       <c r="N32" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- ATUALID</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O32" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="C33" s="22" t="inlineStr">
         <is>
-          <t>DAVI- MAT</t>
+          <t>THOMAZ- HIST</t>
         </is>
       </c>
       <c r="D33" s="47" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="E33" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- OE MAT</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="F33" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="G33" s="45" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="L33" s="16" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="D35" s="29" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>DAVI- MAT</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="H35" s="36" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="J35" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="K35" s="13" t="inlineStr">
@@ -3088,12 +3088,12 @@
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="H36" s="36" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="I36" s="24" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="J36" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="K36" s="13" t="inlineStr">
@@ -3123,12 +3123,12 @@
       </c>
       <c r="N36" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- ATUALID</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="O36" s="48" t="inlineStr">
         <is>
-          <t>BORTOLOTI- PROG</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>ALEXANDRE</t>
         </is>
@@ -4142,7 +4142,7 @@
       <c r="B2" s="52" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>ALINE</t>
         </is>
@@ -4150,7 +4150,7 @@
       <c r="B3" s="53" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>ANDREA</t>
         </is>
@@ -4158,7 +4158,7 @@
       <c r="B4" s="54" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>BAQUETE</t>
         </is>
@@ -4166,7 +4166,7 @@
       <c r="B5" s="55" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>BENEDITA</t>
         </is>
@@ -4174,7 +4174,7 @@
       <c r="B6" s="56" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>BORTOLOTI</t>
         </is>
@@ -4182,7 +4182,7 @@
       <c r="B7" s="57" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
@@ -4190,7 +4190,7 @@
       <c r="B8" s="58" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
@@ -4198,7 +4198,7 @@
       <c r="B9" s="59" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>DAVI</t>
         </is>
@@ -4206,7 +4206,7 @@
       <c r="B10" s="60" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>DINO</t>
         </is>
@@ -4214,7 +4214,7 @@
       <c r="B11" s="61" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>DRIELLI</t>
         </is>
@@ -4222,7 +4222,7 @@
       <c r="B12" s="62" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>EUNICE</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="B13" s="63" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>GERALDO</t>
         </is>
@@ -4238,7 +4238,7 @@
       <c r="B14" s="64" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
@@ -4246,7 +4246,7 @@
       <c r="B15" s="65" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
@@ -4254,7 +4254,7 @@
       <c r="B16" s="66" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
         </is>
@@ -4262,7 +4262,7 @@
       <c r="B17" s="67" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>GISELE</t>
         </is>
@@ -4270,7 +4270,7 @@
       <c r="B18" s="68" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
@@ -4278,7 +4278,7 @@
       <c r="B19" s="69" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
@@ -4286,7 +4286,7 @@
       <c r="B20" s="70" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>LILIANE</t>
         </is>
@@ -4294,7 +4294,7 @@
       <c r="B21" s="71" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>M.EDUARDA</t>
         </is>
@@ -4302,7 +4302,7 @@
       <c r="B22" s="72" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>MARCIA</t>
         </is>
@@ -4310,7 +4310,7 @@
       <c r="B23" s="73" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>MARIANA</t>
         </is>
@@ -4318,7 +4318,7 @@
       <c r="B24" s="74" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>MARINA</t>
         </is>
@@ -4326,7 +4326,7 @@
       <c r="B25" s="75" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
@@ -4334,7 +4334,7 @@
       <c r="B26" s="76" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
@@ -4342,7 +4342,7 @@
       <c r="B27" s="77" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>PAPANONI</t>
         </is>
@@ -4350,7 +4350,7 @@
       <c r="B28" s="78" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
@@ -4358,7 +4358,7 @@
       <c r="B29" s="79" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>RAFAEL</t>
         </is>
@@ -4366,7 +4366,7 @@
       <c r="B30" s="80" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>ROBERTA</t>
         </is>
@@ -4374,7 +4374,7 @@
       <c r="B31" s="81" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>ROMARIO</t>
         </is>
@@ -4382,7 +4382,7 @@
       <c r="B32" s="82" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>SAMIA</t>
         </is>
@@ -4390,7 +4390,7 @@
       <c r="B33" s="83" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>SELMA</t>
         </is>
@@ -4398,7 +4398,7 @@
       <c r="B34" s="84" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>SILVANA</t>
         </is>
@@ -4406,7 +4406,7 @@
       <c r="B35" s="85" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>SILVIA</t>
         </is>
@@ -4414,7 +4414,7 @@
       <c r="B36" s="86" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>SIMARA</t>
         </is>
@@ -4422,7 +4422,7 @@
       <c r="B37" s="87" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>THOMAZ</t>
         </is>
@@ -4430,7 +4430,7 @@
       <c r="B38" s="88" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>VINICIUS</t>
         </is>

</xml_diff>

<commit_message>
Adicionar script de otimização para agendamento de professores
</commit_message>
<xml_diff>
--- a/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
+++ b/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
@@ -146,6 +146,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F77B8F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F76291"/>
       </patternFill>
     </fill>
@@ -196,7 +201,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F77B8F"/>
+        <fgColor rgb="00F788BC"/>
       </patternFill>
     </fill>
     <fill>
@@ -207,6 +212,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007BBCF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009A56F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -222,11 +232,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0088F7B1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F788BC"/>
       </patternFill>
     </fill>
     <fill>
@@ -257,11 +262,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F7DF88"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="009A56F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -394,10 +394,10 @@
     <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -436,7 +436,7 @@
     <xf numFmtId="0" fontId="6" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="32" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -445,13 +445,13 @@
     <xf numFmtId="0" fontId="6" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="38" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -463,7 +463,7 @@
     <xf numFmtId="0" fontId="6" fillId="40" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="41" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="41" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="42" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -473,41 +473,41 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -903,7 +903,7 @@
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="G2" s="17" t="inlineStr">
@@ -933,12 +933,12 @@
       </c>
       <c r="L2" s="22" t="inlineStr">
         <is>
-          <t>DAVI- EFIN</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="M2" s="23" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="N2" s="24" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="O2" s="25" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="H3" s="18" t="inlineStr">
@@ -987,7 +987,7 @@
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
@@ -1002,24 +1002,24 @@
           <t>ANDREA- MATEMÁTICA APL</t>
         </is>
       </c>
-      <c r="L3" s="23" t="inlineStr">
-        <is>
-          <t>DAVI- EFIN</t>
+      <c r="L3" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="M3" s="22" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="N3" s="24" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="O3" s="25" t="inlineStr">
         <is>
-          <t>BORTOLOTI- PROG</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1028,12 +1028,12 @@
       <c r="B4" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C4" s="26" t="inlineStr">
-        <is>
-          <t>ROMARIO- ED FÍSICA</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>THOMAZ- HIST</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
@@ -1058,9 +1058,9 @@
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
-        <is>
-          <t>MARCIA- ARTE</t>
+      <c r="I4" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J4" s="21" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
+          <t>MARINA- REDAÇÃO</t>
+        </is>
+      </c>
+      <c r="O4" s="29" t="inlineStr">
+        <is>
           <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
-      <c r="O4" s="28" t="inlineStr">
-        <is>
-          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1099,12 @@
       <c r="B5" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>ROMARIO- ED FÍSICA</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
@@ -1151,17 +1151,17 @@
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
+          <t>GERALDO- MAT</t>
+        </is>
+      </c>
+      <c r="N5" s="22" t="inlineStr">
+        <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="O5" s="29" t="inlineStr">
+        <is>
           <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
-      <c r="N5" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="O5" s="28" t="inlineStr">
-        <is>
-          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       <c r="B7" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
@@ -1201,14 +1201,14 @@
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="E7" s="30" t="inlineStr">
+      <c r="E7" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>PAPANONI- ED. FINAN</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="K7" s="18" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="L7" s="19" t="inlineStr">
@@ -1246,9 +1246,9 @@
           <t>ANDREA- GESTÃO DE OPER.</t>
         </is>
       </c>
-      <c r="N7" s="28" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
+      <c r="N7" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O7" s="22" t="inlineStr">
@@ -1262,7 +1262,7 @@
       <c r="B8" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
@@ -1272,41 +1272,41 @@
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr">
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>DRIELLI- CARREIRA E COMP</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="J8" s="20" t="inlineStr">
-        <is>
-          <t>DRIELLI- CARREIRA E COMP</t>
-        </is>
-      </c>
-      <c r="K8" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
@@ -1317,9 +1317,9 @@
           <t>ANDREA- GESTÃO DE OPER.</t>
         </is>
       </c>
-      <c r="N8" s="28" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
+      <c r="N8" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O8" s="22" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -1352,54 +1352,54 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>PAPANONI- ED. FINAN</t>
-        </is>
-      </c>
-      <c r="G9" s="29" t="inlineStr">
-        <is>
-          <t>ALINE- FILOSOFIA</t>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="G9" s="30" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="H9" s="22" t="inlineStr">
         <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="J9" s="32" t="inlineStr">
+        <is>
+          <t>MAT APLICADA</t>
+        </is>
+      </c>
+      <c r="K9" s="33" t="inlineStr">
+        <is>
+          <t>INTRODUÇÃO ADM</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="I9" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="J9" s="31" t="inlineStr">
-        <is>
-          <t>MAT APLICADA</t>
-        </is>
-      </c>
-      <c r="K9" s="32" t="inlineStr">
-        <is>
-          <t>INTRODUÇÃO ADM</t>
-        </is>
-      </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="M9" s="28" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="N9" s="33" t="inlineStr">
+      <c r="M9" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
+        </is>
+      </c>
+      <c r="N9" s="34" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -1425,52 +1425,52 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="G10" s="30" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="G10" s="29" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="H10" s="22" t="inlineStr">
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="J10" s="32" t="inlineStr">
+        <is>
+          <t>MAT APLICADA</t>
+        </is>
+      </c>
+      <c r="K10" s="33" t="inlineStr">
+        <is>
+          <t>INTRODUÇÃO ADM</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="M10" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
+        </is>
+      </c>
+      <c r="N10" s="34" t="inlineStr">
+        <is>
+          <t>SAMIA- AP SOC</t>
+        </is>
+      </c>
+      <c r="O10" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="J10" s="31" t="inlineStr">
-        <is>
-          <t>MAT APLICADA</t>
-        </is>
-      </c>
-      <c r="K10" s="32" t="inlineStr">
-        <is>
-          <t>INTRODUÇÃO ADM</t>
-        </is>
-      </c>
-      <c r="L10" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="M10" s="28" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
-      <c r="N10" s="33" t="inlineStr">
-        <is>
-          <t>SAMIA- AP SOC</t>
-        </is>
-      </c>
-      <c r="O10" s="24" t="inlineStr">
-        <is>
-          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -1479,17 +1479,17 @@
       <c r="B11" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>DAVI- MAT</t>
-        </is>
-      </c>
-      <c r="E11" s="30" t="inlineStr">
+          <t>MARINA- OE PORT</t>
+        </is>
+      </c>
+      <c r="E11" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
@@ -1501,32 +1501,32 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="H11" s="29" t="inlineStr">
+          <t>SILVANA- RED</t>
+        </is>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
         <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="I11" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- EFIN</t>
-        </is>
-      </c>
-      <c r="J11" s="32" t="inlineStr">
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="J11" s="33" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
       </c>
-      <c r="K11" s="31" t="inlineStr">
+      <c r="K11" s="32" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
       </c>
       <c r="L11" s="22" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="M11" s="17" t="inlineStr">
@@ -1534,14 +1534,14 @@
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="N11" s="33" t="inlineStr">
+      <c r="N11" s="34" t="inlineStr">
         <is>
           <t>SAMIA- AP SOC</t>
         </is>
       </c>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>ALINE- SOC</t>
         </is>
       </c>
     </row>
@@ -1550,12 +1550,12 @@
       <c r="B12" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="C12" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="D12" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
@@ -1575,39 +1575,39 @@
           <t>SILVANA- RED</t>
         </is>
       </c>
-      <c r="H12" s="29" t="inlineStr">
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>INTRODUÇÃO ADM</t>
+        </is>
+      </c>
+      <c r="K12" s="32" t="inlineStr">
+        <is>
+          <t>MAT APLICADA</t>
+        </is>
+      </c>
+      <c r="L12" s="34" t="inlineStr">
+        <is>
+          <t>SAMIA- ARTE E MÍDIA</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="N12" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="I12" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="J12" s="32" t="inlineStr">
-        <is>
-          <t>INTRODUÇÃO ADM</t>
-        </is>
-      </c>
-      <c r="K12" s="31" t="inlineStr">
-        <is>
-          <t>MAT APLICADA</t>
-        </is>
-      </c>
-      <c r="L12" s="33" t="inlineStr">
-        <is>
-          <t>SAMIA- ARTE E MÍDIA</t>
-        </is>
-      </c>
-      <c r="M12" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="N12" s="22" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="O12" s="18" t="inlineStr">
@@ -1647,12 +1647,12 @@
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D14" s="33" t="inlineStr">
+      <c r="D14" s="34" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
-      <c r="E14" s="27" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
@@ -1664,20 +1664,20 @@
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="H14" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I14" s="29" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="J14" s="34" t="inlineStr">
+      <c r="J14" s="35" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
@@ -1692,7 +1692,7 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="M14" s="35" t="inlineStr">
+      <c r="M14" s="36" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="O14" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       <c r="B15" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>THOMAZ- HIST</t>
         </is>
@@ -1723,7 +1723,7 @@
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="E15" s="27" t="inlineStr">
+      <c r="E15" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="H15" s="24" t="inlineStr">
@@ -1743,9 +1743,9 @@
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="I15" s="29" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
+      <c r="I15" s="30" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="J15" s="25" t="inlineStr">
@@ -1753,7 +1753,7 @@
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="K15" s="34" t="inlineStr">
+      <c r="K15" s="35" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
@@ -1763,7 +1763,7 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="M15" s="35" t="inlineStr">
+      <c r="M15" s="36" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="O15" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
     </row>
@@ -1798,59 +1798,59 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="E16" s="33" t="inlineStr">
+      <c r="E16" s="34" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="G16" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="K16" s="35" t="inlineStr">
+        <is>
+          <t>CARREIRA E COMP</t>
+        </is>
+      </c>
+      <c r="L16" s="26" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="J16" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="K16" s="34" t="inlineStr">
-        <is>
-          <t>CARREIRA E COMP</t>
-        </is>
-      </c>
-      <c r="L16" s="36" t="inlineStr">
-        <is>
-          <t>ALINE- ORATÓRIA</t>
-        </is>
-      </c>
       <c r="M16" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="N16" s="28" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
+      <c r="N16" s="37" t="inlineStr">
+        <is>
+          <t>SIMARA- OE LP</t>
         </is>
       </c>
       <c r="O16" s="23" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="F17" s="24" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="G17" s="22" t="inlineStr">
         <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
           <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="I17" s="36" t="inlineStr">
-        <is>
-          <t>MARCIA- ARTE</t>
+      <c r="I17" s="18" t="inlineStr">
+        <is>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr">
@@ -1899,12 +1899,12 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="K17" s="34" t="inlineStr">
+      <c r="K17" s="35" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
       </c>
-      <c r="L17" s="33" t="inlineStr">
+      <c r="L17" s="34" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="N17" s="23" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="O17" s="28" t="inlineStr">
-        <is>
-          <t>VINICIUS- AP QUIM</t>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="O17" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       <c r="B18" s="3" t="n">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C18" s="30" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
@@ -1940,54 +1940,54 @@
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="E18" s="27" t="inlineStr">
+      <c r="E18" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
-        </is>
-      </c>
-      <c r="I18" s="36" t="inlineStr">
-        <is>
-          <t>ALINE- FILOSOFIA</t>
-        </is>
-      </c>
-      <c r="J18" s="33" t="inlineStr">
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="J18" s="34" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="K18" s="37" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
+      <c r="K18" s="38" t="inlineStr">
+        <is>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="L18" s="22" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="M18" s="28" t="inlineStr">
+          <t>DAVI- EFIN</t>
+        </is>
+      </c>
+      <c r="M18" s="29" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="N18" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- ATUALID</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="O18" s="13" t="inlineStr">
@@ -2001,7 +2001,7 @@
       <c r="B19" s="3" t="n">
         <v>0.3958333333333333</v>
       </c>
-      <c r="C19" s="30" t="inlineStr">
+      <c r="C19" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
@@ -2011,14 +2011,14 @@
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="E19" s="27" t="inlineStr">
+      <c r="E19" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
@@ -2031,32 +2031,32 @@
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="I19" s="38" t="inlineStr">
+      <c r="I19" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="J19" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="K19" s="37" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
+      <c r="J19" s="40" t="inlineStr">
+        <is>
+          <t>RAFAEL- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="K19" s="38" t="inlineStr">
+        <is>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="L19" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="M19" s="39" t="inlineStr">
+          <t>DAVI- EFIN</t>
+        </is>
+      </c>
+      <c r="M19" s="41" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
       </c>
-      <c r="N19" s="33" t="inlineStr">
+      <c r="N19" s="34" t="inlineStr">
         <is>
           <t>SAMIA- AP FIL</t>
         </is>
@@ -2098,12 +2098,12 @@
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D21" s="27" t="inlineStr">
+      <c r="D21" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="25" t="inlineStr">
         <is>
           <t>GERALDO- OE MAT</t>
         </is>
@@ -2113,9 +2113,9 @@
           <t>SILVANA- RED</t>
         </is>
       </c>
-      <c r="G21" s="36" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
+      <c r="G21" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
@@ -2123,14 +2123,14 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="I21" s="38" t="inlineStr">
+      <c r="I21" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
       <c r="J21" s="18" t="inlineStr">
         <is>
-          <t>RAFAEL- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="K21" s="17" t="inlineStr">
@@ -2140,22 +2140,22 @@
       </c>
       <c r="L21" s="18" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="M21" s="39" t="inlineStr">
+          <t>ALINE- ORATÓRIA</t>
+        </is>
+      </c>
+      <c r="M21" s="41" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
       </c>
-      <c r="N21" s="25" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
       <c r="O21" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
     </row>
@@ -2164,29 +2164,29 @@
       <c r="B22" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>THOMAZ- HIST</t>
         </is>
       </c>
-      <c r="D22" s="27" t="inlineStr">
+      <c r="D22" s="28" t="inlineStr">
         <is>
           <t>SELMA- CIÊN</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>GERALDO- OE MAT</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="G22" s="36" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>SILVANA- RED</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="J22" s="18" t="inlineStr">
         <is>
-          <t>BENEDITA- GEO</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="K22" s="17" t="inlineStr">
@@ -2214,19 +2214,19 @@
           <t>ALINE- ORATÓRIA</t>
         </is>
       </c>
-      <c r="M22" s="39" t="inlineStr">
+      <c r="M22" s="41" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
       </c>
       <c r="N22" s="25" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
     </row>
@@ -2254,54 +2254,54 @@
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="F23" s="38" t="inlineStr">
+      <c r="F23" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- EFIN</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="J23" s="17" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
       <c r="K23" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="L23" s="33" t="inlineStr">
+      <c r="L23" s="34" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="M23" s="40" t="inlineStr">
+      <c r="M23" s="42" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
       </c>
-      <c r="N23" s="28" t="inlineStr">
-        <is>
-          <t>SIMARA- OE LP</t>
-        </is>
-      </c>
-      <c r="O23" s="36" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
+      <c r="N23" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
+        </is>
+      </c>
+      <c r="O23" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -2312,10 +2312,10 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
-        </is>
-      </c>
-      <c r="D24" s="22" t="inlineStr">
+          <t>MARINA- PORT</t>
+        </is>
+      </c>
+      <c r="D24" s="30" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
@@ -2325,14 +2325,14 @@
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="F24" s="38" t="inlineStr">
+      <c r="F24" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -2342,10 +2342,10 @@
       </c>
       <c r="I24" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="J24" s="33" t="inlineStr">
+          <t>SILVIA- EFIN</t>
+        </is>
+      </c>
+      <c r="J24" s="34" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
@@ -2355,22 +2355,22 @@
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="L24" s="36" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="M24" s="40" t="inlineStr">
+      <c r="L24" s="23" t="inlineStr">
+        <is>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="M24" s="42" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
       </c>
       <c r="N24" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- ATUALID</t>
-        </is>
-      </c>
-      <c r="O24" s="28" t="inlineStr">
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="O24" s="29" t="inlineStr">
         <is>
           <t>M.EDUARDA- PORT</t>
         </is>
@@ -2383,32 +2383,32 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
+          <t>ROMARIO- ED FÍSICA</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>ROMARIO- ED FÍSICA</t>
-        </is>
-      </c>
-      <c r="E25" s="30" t="inlineStr">
+      <c r="E25" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F25" s="33" t="inlineStr">
+      <c r="F25" s="34" t="inlineStr">
         <is>
           <t>SAMIA- ARTE</t>
         </is>
       </c>
-      <c r="G25" s="38" t="inlineStr">
+      <c r="G25" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="I25" s="16" t="inlineStr">
@@ -2416,34 +2416,34 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="J25" s="37" t="inlineStr">
+      <c r="J25" s="38" t="inlineStr">
+        <is>
+          <t>BENEDITA- GEO</t>
+        </is>
+      </c>
+      <c r="K25" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="L25" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="K25" s="36" t="inlineStr">
-        <is>
-          <t>BENEDITA- GEO</t>
-        </is>
-      </c>
-      <c r="L25" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="M25" s="41" t="inlineStr">
+      <c r="M25" s="43" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
         </is>
       </c>
-      <c r="N25" s="42" t="inlineStr">
-        <is>
-          <t>MARINA- REDAÇÃO</t>
+      <c r="N25" s="37" t="inlineStr">
+        <is>
+          <t>SIMARA- OE LP</t>
         </is>
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="D26" s="22" t="inlineStr">
@@ -2467,19 +2467,19 @@
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="F26" s="33" t="inlineStr">
+      <c r="F26" s="34" t="inlineStr">
         <is>
           <t>SAMIA- ARTE</t>
         </is>
       </c>
-      <c r="G26" s="38" t="inlineStr">
+      <c r="G26" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="I26" s="16" t="inlineStr">
@@ -2487,34 +2487,34 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="J26" s="37" t="inlineStr">
+      <c r="J26" s="38" t="inlineStr">
+        <is>
+          <t>BENEDITA- GEO</t>
+        </is>
+      </c>
+      <c r="K26" s="26" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="K26" s="36" t="inlineStr">
+      <c r="L26" s="18" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="L26" s="18" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="M26" s="43" t="inlineStr">
+      <c r="M26" s="44" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
       </c>
-      <c r="N26" s="42" t="inlineStr">
-        <is>
-          <t>SIMARA- OE LP</t>
+      <c r="N26" s="29" t="inlineStr">
+        <is>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
           <t>DAVI- MAT</t>
         </is>
       </c>
-      <c r="D28" s="30" t="inlineStr">
+      <c r="D28" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- OE MAT</t>
         </is>
@@ -2559,9 +2559,9 @@
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="F28" s="44" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
+      <c r="F28" s="45" t="inlineStr">
+        <is>
+          <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
@@ -2569,19 +2569,19 @@
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="H28" s="38" t="inlineStr">
+      <c r="H28" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="J28" s="36" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="J28" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="K28" s="16" t="inlineStr">
@@ -2589,17 +2589,17 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="L28" s="45" t="inlineStr">
+      <c r="L28" s="46" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
       </c>
-      <c r="M28" s="46" t="inlineStr">
+      <c r="M28" s="47" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="N28" s="47" t="inlineStr">
+      <c r="N28" s="48" t="inlineStr">
         <is>
           <t>DINO- AP GEO</t>
         </is>
@@ -2625,14 +2625,14 @@
           <t>EUNICE- HIST</t>
         </is>
       </c>
-      <c r="E29" s="30" t="inlineStr">
+      <c r="E29" s="31" t="inlineStr">
         <is>
           <t>BAQUETE- MAT</t>
         </is>
       </c>
-      <c r="F29" s="44" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
+      <c r="F29" s="45" t="inlineStr">
+        <is>
+          <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
@@ -2640,19 +2640,19 @@
           <t>SILVIA- MAT</t>
         </is>
       </c>
-      <c r="H29" s="38" t="inlineStr">
+      <c r="H29" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="I29" s="18" t="inlineStr">
+      <c r="I29" s="19" t="inlineStr">
         <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="J29" s="36" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
+      <c r="J29" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
@@ -2660,24 +2660,24 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="L29" s="45" t="inlineStr">
+      <c r="L29" s="46" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
       </c>
-      <c r="M29" s="46" t="inlineStr">
+      <c r="M29" s="47" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="N29" s="47" t="inlineStr">
+      <c r="N29" s="48" t="inlineStr">
         <is>
           <t>DINO- AP GEO</t>
         </is>
       </c>
-      <c r="O29" s="48" t="inlineStr">
-        <is>
-          <t>ALINE- SOC</t>
+      <c r="O29" s="49" t="inlineStr">
+        <is>
+          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       <c r="B30" s="3" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C30" s="34" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
@@ -2700,7 +2700,7 @@
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="E30" s="47" t="inlineStr">
+      <c r="E30" s="48" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
@@ -2715,17 +2715,17 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="H30" s="45" t="inlineStr">
+      <c r="H30" s="46" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>SILVIA- EFIN</t>
-        </is>
-      </c>
-      <c r="J30" s="49" t="inlineStr">
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
         </is>
@@ -2735,12 +2735,12 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="L30" s="38" t="inlineStr">
+      <c r="L30" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="M30" s="46" t="inlineStr">
+      <c r="M30" s="47" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>VINICIUS- AP QUIM</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
@@ -2771,14 +2771,14 @@
           <t>ROBERTA- PORT</t>
         </is>
       </c>
-      <c r="E31" s="47" t="inlineStr">
+      <c r="E31" s="48" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
       <c r="F31" s="22" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="G31" s="13" t="inlineStr">
@@ -2786,14 +2786,14 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="H31" s="45" t="inlineStr">
+      <c r="H31" s="46" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="J31" s="16" t="inlineStr">
@@ -2801,29 +2801,29 @@
           <t>SILVANA- PORT</t>
         </is>
       </c>
-      <c r="K31" s="33" t="inlineStr">
+      <c r="K31" s="34" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
         </is>
       </c>
-      <c r="L31" s="38" t="inlineStr">
+      <c r="L31" s="39" t="inlineStr">
         <is>
           <t>MARIANA- GEO</t>
         </is>
       </c>
-      <c r="M31" s="43" t="inlineStr">
+      <c r="M31" s="44" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
       </c>
-      <c r="N31" s="24" t="inlineStr">
+      <c r="N31" s="25" t="inlineStr">
         <is>
           <t>GERALDO- MAT</t>
         </is>
       </c>
-      <c r="O31" s="36" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
+      <c r="O31" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -2834,67 +2834,67 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
-        </is>
-      </c>
-      <c r="D32" s="47" t="inlineStr">
+          <t>MARINA- PORT</t>
+        </is>
+      </c>
+      <c r="D32" s="48" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="E32" s="25" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="F32" s="36" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>ROMARIO- ED FÍSICA</t>
+        </is>
+      </c>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="G32" s="46" t="inlineStr">
+        <is>
+          <t>LILIANE- ED. FINAN</t>
+        </is>
+      </c>
+      <c r="H32" s="30" t="inlineStr">
+        <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="I32" s="22" t="inlineStr">
+        <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="K32" s="34" t="inlineStr">
+        <is>
+          <t>SAMIA- SOC</t>
+        </is>
+      </c>
+      <c r="L32" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="M32" s="44" t="inlineStr">
+        <is>
+          <t>PROJETO MULTI</t>
+        </is>
+      </c>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- ATUALID</t>
+        </is>
+      </c>
+      <c r="O32" s="24" t="inlineStr">
         <is>
           <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="G32" s="45" t="inlineStr">
-        <is>
-          <t>LILIANE- ED. FINAN</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>MARCIA- ARTE</t>
-        </is>
-      </c>
-      <c r="I32" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="J32" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="K32" s="33" t="inlineStr">
-        <is>
-          <t>SAMIA- SOC</t>
-        </is>
-      </c>
-      <c r="L32" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="M32" s="43" t="inlineStr">
-        <is>
-          <t>PROJETO MULTI</t>
-        </is>
-      </c>
-      <c r="N32" s="17" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
-      <c r="O32" s="24" t="inlineStr">
-        <is>
-          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -2905,25 +2905,25 @@
       </c>
       <c r="C33" s="22" t="inlineStr">
         <is>
-          <t>THOMAZ- HIST</t>
-        </is>
-      </c>
-      <c r="D33" s="47" t="inlineStr">
+          <t>DAVI- MAT</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
       <c r="E33" s="25" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
-        </is>
-      </c>
-      <c r="F33" s="36" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="G33" s="45" t="inlineStr">
+          <t>GERALDO- OE MAT</t>
+        </is>
+      </c>
+      <c r="F33" s="26" t="inlineStr">
+        <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="G33" s="46" t="inlineStr">
         <is>
           <t>LILIANE- ED. FINAN</t>
         </is>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>BENEDITA- GEO</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="L33" s="16" t="inlineStr">
@@ -2963,7 +2963,7 @@
           <t>SILVIA- OE MAT</t>
         </is>
       </c>
-      <c r="O33" s="33" t="inlineStr">
+      <c r="O33" s="34" t="inlineStr">
         <is>
           <t>SAMIA- PV</t>
         </is>
@@ -2995,12 +2995,12 @@
       <c r="B35" s="3" t="n">
         <v>0.4444444444444444</v>
       </c>
-      <c r="C35" s="47" t="inlineStr">
+      <c r="C35" s="48" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
       </c>
-      <c r="D35" s="29" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>DAVI- MAT</t>
         </is>
@@ -3017,10 +3017,10 @@
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="H35" s="36" t="inlineStr">
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="H35" s="26" t="inlineStr">
         <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="J35" s="25" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K35" s="13" t="inlineStr">
@@ -3040,7 +3040,7 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="L35" s="45" t="inlineStr">
+      <c r="L35" s="46" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
@@ -3050,7 +3050,7 @@
           <t>MARKETING</t>
         </is>
       </c>
-      <c r="N35" s="33" t="inlineStr">
+      <c r="N35" s="34" t="inlineStr">
         <is>
           <t>SAMIA- AP FILO</t>
         </is>
@@ -3066,7 +3066,7 @@
       <c r="B36" s="3" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C36" s="47" t="inlineStr">
+      <c r="C36" s="48" t="inlineStr">
         <is>
           <t>DINO- GEO</t>
         </is>
@@ -3076,7 +3076,7 @@
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="E36" s="29" t="inlineStr">
+      <c r="E36" s="30" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
@@ -3088,10 +3088,10 @@
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="H36" s="36" t="inlineStr">
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="H36" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
         </is>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="J36" s="25" t="inlineStr">
         <is>
-          <t>BENEDITA- GEO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K36" s="13" t="inlineStr">
@@ -3111,7 +3111,7 @@
           <t>ALEXANDRE- ING</t>
         </is>
       </c>
-      <c r="L36" s="45" t="inlineStr">
+      <c r="L36" s="46" t="inlineStr">
         <is>
           <t>LILIANE- MAT</t>
         </is>
@@ -3123,12 +3123,12 @@
       </c>
       <c r="N36" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="O36" s="48" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>EUNICE- ATUALID</t>
+        </is>
+      </c>
+      <c r="O36" s="49" t="inlineStr">
+        <is>
+          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ALEXANDRE</t>
         </is>
@@ -4142,7 +4142,7 @@
       <c r="B2" s="52" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ALINE</t>
         </is>
@@ -4150,7 +4150,7 @@
       <c r="B3" s="53" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>ANDREA</t>
         </is>
@@ -4158,7 +4158,7 @@
       <c r="B4" s="54" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>BAQUETE</t>
         </is>
@@ -4166,7 +4166,7 @@
       <c r="B5" s="55" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>BENEDITA</t>
         </is>
@@ -4174,7 +4174,7 @@
       <c r="B6" s="56" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>BORTOLOTI</t>
         </is>
@@ -4182,7 +4182,7 @@
       <c r="B7" s="57" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
@@ -4190,7 +4190,7 @@
       <c r="B8" s="58" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="0" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
@@ -4198,7 +4198,7 @@
       <c r="B9" s="59" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>DAVI</t>
         </is>
@@ -4206,7 +4206,7 @@
       <c r="B10" s="60" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>DINO</t>
         </is>
@@ -4214,7 +4214,7 @@
       <c r="B11" s="61" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="0" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>DRIELLI</t>
         </is>
@@ -4222,7 +4222,7 @@
       <c r="B12" s="62" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="0" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>EUNICE</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="B13" s="63" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="0" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>GERALDO</t>
         </is>
@@ -4238,7 +4238,7 @@
       <c r="B14" s="64" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="0" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
@@ -4246,7 +4246,7 @@
       <c r="B15" s="65" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="0" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
@@ -4254,7 +4254,7 @@
       <c r="B16" s="66" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="0" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
         </is>
@@ -4262,7 +4262,7 @@
       <c r="B17" s="67" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="0" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>GISELE</t>
         </is>
@@ -4270,7 +4270,7 @@
       <c r="B18" s="68" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="0" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
@@ -4278,7 +4278,7 @@
       <c r="B19" s="69" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="0" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
@@ -4286,7 +4286,7 @@
       <c r="B20" s="70" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="0" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>LILIANE</t>
         </is>
@@ -4294,7 +4294,7 @@
       <c r="B21" s="71" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="0" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>M.EDUARDA</t>
         </is>
@@ -4302,7 +4302,7 @@
       <c r="B22" s="72" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="0" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>MARCIA</t>
         </is>
@@ -4310,7 +4310,7 @@
       <c r="B23" s="73" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="0" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>MARIANA</t>
         </is>
@@ -4318,7 +4318,7 @@
       <c r="B24" s="74" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="0" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>MARINA</t>
         </is>
@@ -4326,7 +4326,7 @@
       <c r="B25" s="75" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="0" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
@@ -4334,7 +4334,7 @@
       <c r="B26" s="76" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="0" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
@@ -4342,7 +4342,7 @@
       <c r="B27" s="77" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="0" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>PAPANONI</t>
         </is>
@@ -4350,7 +4350,7 @@
       <c r="B28" s="78" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="0" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
@@ -4358,7 +4358,7 @@
       <c r="B29" s="79" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="0" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>RAFAEL</t>
         </is>
@@ -4366,7 +4366,7 @@
       <c r="B30" s="80" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="0" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>ROBERTA</t>
         </is>
@@ -4374,7 +4374,7 @@
       <c r="B31" s="81" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="0" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>ROMARIO</t>
         </is>
@@ -4382,7 +4382,7 @@
       <c r="B32" s="82" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="0" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>SAMIA</t>
         </is>
@@ -4390,7 +4390,7 @@
       <c r="B33" s="83" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="0" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>SELMA</t>
         </is>
@@ -4398,7 +4398,7 @@
       <c r="B34" s="84" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="0" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>SILVANA</t>
         </is>
@@ -4406,7 +4406,7 @@
       <c r="B35" s="85" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="0" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>SILVIA</t>
         </is>
@@ -4414,7 +4414,7 @@
       <c r="B36" s="86" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="0" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>SIMARA</t>
         </is>
@@ -4422,7 +4422,7 @@
       <c r="B37" s="87" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="0" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>THOMAZ</t>
         </is>
@@ -4430,7 +4430,7 @@
       <c r="B38" s="88" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="0" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>VINICIUS</t>
         </is>

</xml_diff>

<commit_message>
Atualizar arquivo Excel com novos dados de agendamento
</commit_message>
<xml_diff>
--- a/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
+++ b/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="I3" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="J3" s="20" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="H4" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="I4" s="26" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="O4" s="29" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>THOMAZ- HIST</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
           <t>MARINA- REDAÇÃO</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="J5" s="21" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G9" s="30" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G10" s="30" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="E11" s="31" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="I11" s="24" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>ALINE- SOC</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1572,12 @@
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="H12" s="30" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="I12" s="24" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="O12" s="18" t="inlineStr">
         <is>
-          <t>ALINE- SOC</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="H14" s="24" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="I14" s="30" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="J14" s="35" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="K14" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="L14" s="16" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="O14" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="H15" s="24" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="I15" s="30" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J15" s="25" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -1810,14 +1810,14 @@
       </c>
       <c r="G16" s="22" t="inlineStr">
         <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- FILOSOFIA</t>
-        </is>
-      </c>
       <c r="I16" s="17" t="inlineStr">
         <is>
           <t>EUNICE- HIST</t>
@@ -1840,17 +1840,17 @@
       </c>
       <c r="M16" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="N16" s="37" t="inlineStr">
         <is>
-          <t>SIMARA- OE LP</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O16" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="G17" s="22" t="inlineStr">
         <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
           <t>DAVI- FÍSICA</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- FILOSOFIA</t>
-        </is>
-      </c>
       <c r="I17" s="18" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr">
@@ -1937,47 +1937,47 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
+          <t>ROMARIO- ED FÍSICA</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>SELMA- CIÊN</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="H18" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="inlineStr">
+        <is>
           <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
-      <c r="E18" s="28" t="inlineStr">
-        <is>
-          <t>SELMA- CIÊN</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="J18" s="34" t="inlineStr">
+        <is>
+          <t>SAMIA- SOC</t>
+        </is>
+      </c>
+      <c r="K18" s="38" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="H18" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I18" s="26" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="J18" s="34" t="inlineStr">
-        <is>
-          <t>SAMIA- SOC</t>
-        </is>
-      </c>
-      <c r="K18" s="38" t="inlineStr">
-        <is>
-          <t>BENEDITA- GEO</t>
-        </is>
-      </c>
       <c r="L18" s="22" t="inlineStr">
         <is>
-          <t>DAVI- EFIN</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="M18" s="29" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="E19" s="28" t="inlineStr">
@@ -2018,37 +2018,37 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
+          <t>GISELE- ED. FÍSICA</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="I19" s="39" t="inlineStr">
+        <is>
+          <t>MARIANA- GEO</t>
+        </is>
+      </c>
+      <c r="J19" s="40" t="inlineStr">
+        <is>
+          <t>GERALDO- MAT</t>
+        </is>
+      </c>
+      <c r="K19" s="38" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="H19" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I19" s="39" t="inlineStr">
-        <is>
-          <t>MARIANA- GEO</t>
-        </is>
-      </c>
-      <c r="J19" s="40" t="inlineStr">
-        <is>
-          <t>RAFAEL- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="K19" s="38" t="inlineStr">
-        <is>
-          <t>BENEDITA- GEO</t>
-        </is>
-      </c>
       <c r="L19" s="22" t="inlineStr">
         <is>
-          <t>DAVI- EFIN</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="M19" s="41" t="inlineStr">
@@ -2110,39 +2110,39 @@
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="G21" s="26" t="inlineStr">
         <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="I21" s="39" t="inlineStr">
+        <is>
+          <t>MARIANA- GEO</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="inlineStr">
+        <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="L21" s="18" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="I21" s="39" t="inlineStr">
-        <is>
-          <t>MARIANA- GEO</t>
-        </is>
-      </c>
-      <c r="J21" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="K21" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="L21" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- ORATÓRIA</t>
-        </is>
-      </c>
       <c r="M21" s="41" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
@@ -2150,12 +2150,12 @@
       </c>
       <c r="N21" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="O21" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>THOMAZ- HIST</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D22" s="28" t="inlineStr">
@@ -2181,39 +2181,39 @@
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- RED</t>
+          <t>SILVANA- PORT</t>
         </is>
       </c>
       <c r="G22" s="26" t="inlineStr">
         <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="I22" s="22" t="inlineStr">
+        <is>
+          <t>DAVI- FÍSICA</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="L22" s="18" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="I22" s="22" t="inlineStr">
-        <is>
-          <t>DAVI- FÍSICA</t>
-        </is>
-      </c>
-      <c r="J22" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="L22" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- ORATÓRIA</t>
-        </is>
-      </c>
       <c r="M22" s="41" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
@@ -2221,12 +2221,12 @@
       </c>
       <c r="N22" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
@@ -2261,29 +2261,29 @@
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
+          <t>MARCIA- ARTE</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="K23" s="25" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- EFIN</t>
-        </is>
-      </c>
-      <c r="J23" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="K23" s="25" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
-        </is>
-      </c>
       <c r="L23" s="34" t="inlineStr">
         <is>
           <t>SAMIA- SOC</t>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="O23" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- AP QUIM</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -2312,52 +2312,52 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D24" s="30" t="inlineStr">
         <is>
+          <t>DAVI- MAT</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>ROBERTA- PORT</t>
+        </is>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>MARIANA- GEO</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
-        <is>
-          <t>ROBERTA- PORT</t>
-        </is>
-      </c>
-      <c r="F24" s="39" t="inlineStr">
-        <is>
-          <t>MARIANA- GEO</t>
-        </is>
-      </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="J24" s="34" t="inlineStr">
+        <is>
+          <t>SAMIA- SOC</t>
+        </is>
+      </c>
+      <c r="K24" s="25" t="inlineStr">
         <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="H24" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="I24" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- EFIN</t>
-        </is>
-      </c>
-      <c r="J24" s="34" t="inlineStr">
-        <is>
-          <t>SAMIA- SOC</t>
-        </is>
-      </c>
-      <c r="K24" s="25" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
-        </is>
-      </c>
       <c r="L24" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="M24" s="42" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="O24" s="29" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D25" s="22" t="inlineStr">
@@ -2418,19 +2418,19 @@
       </c>
       <c r="J25" s="38" t="inlineStr">
         <is>
-          <t>BENEDITA- GEO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K25" s="26" t="inlineStr">
         <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="L25" s="18" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="L25" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
       <c r="M25" s="43" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
@@ -2438,12 +2438,12 @@
       </c>
       <c r="N25" s="37" t="inlineStr">
         <is>
-          <t>SIMARA- OE LP</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>THOMAZ- HIST</t>
         </is>
       </c>
       <c r="D26" s="22" t="inlineStr">
@@ -2489,19 +2489,19 @@
       </c>
       <c r="J26" s="38" t="inlineStr">
         <is>
-          <t>BENEDITA- GEO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K26" s="26" t="inlineStr">
         <is>
+          <t>ALINE- BIO</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
-      <c r="L26" s="18" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
       <c r="M26" s="44" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
     </row>
@@ -2556,12 +2556,12 @@
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
       <c r="F28" s="45" t="inlineStr">
         <is>
-          <t>PAPANONI- ED. FINAN</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
@@ -2576,12 +2576,12 @@
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J28" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K28" s="16" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="F29" s="45" t="inlineStr">
         <is>
-          <t>PAPANONI- ED. FINAN</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="J29" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="O29" s="49" t="inlineStr">
         <is>
-          <t>BORTOLOTI- PROG</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J30" s="17" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="J31" s="16" t="inlineStr">
@@ -2818,12 +2818,12 @@
       </c>
       <c r="N31" s="25" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="O31" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- AP QUIM</t>
+          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>MARINA- PORT</t>
+          <t>MARINA- OE LP</t>
         </is>
       </c>
       <c r="D32" s="48" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>GERALDO- OE MAT</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>ALINE- FILOSOFIA</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
       <c r="G32" s="46" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="H32" s="30" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="I32" s="22" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="N32" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- ATUALID</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O32" s="24" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="F33" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="G33" s="46" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="I33" s="17" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="K33" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="L33" s="16" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="N33" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- OE MAT</t>
+          <t>SILVIA- MAT</t>
         </is>
       </c>
       <c r="O33" s="34" t="inlineStr">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
@@ -3017,12 +3017,12 @@
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="H35" s="26" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="I35" s="24" t="inlineStr">
@@ -3073,24 +3073,24 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
+          <t>ROMARIO- ED FÍSICA</t>
+        </is>
+      </c>
+      <c r="E36" s="30" t="inlineStr">
+        <is>
           <t>MARINA- OE PORT</t>
         </is>
       </c>
-      <c r="E36" s="30" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>SILVANA- PORT</t>
+        </is>
+      </c>
+      <c r="G36" s="23" t="inlineStr">
         <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="F36" s="16" t="inlineStr">
-        <is>
-          <t>SILVANA- PORT</t>
-        </is>
-      </c>
-      <c r="G36" s="23" t="inlineStr">
-        <is>
-          <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
       <c r="H36" s="22" t="inlineStr">
         <is>
           <t>DAVI- FÍSICA</t>
@@ -3123,12 +3123,12 @@
       </c>
       <c r="N36" s="17" t="inlineStr">
         <is>
-          <t>EUNICE- ATUALID</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
       <c r="O36" s="49" t="inlineStr">
         <is>
-          <t>BORTOLOTI- PROG</t>
+          <t>EUNICE- HIST</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>ALEXANDRE</t>
         </is>
@@ -4142,7 +4142,7 @@
       <c r="B2" s="52" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>ALINE</t>
         </is>
@@ -4150,7 +4150,7 @@
       <c r="B3" s="53" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>ANDREA</t>
         </is>
@@ -4158,7 +4158,7 @@
       <c r="B4" s="54" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>BAQUETE</t>
         </is>
@@ -4166,7 +4166,7 @@
       <c r="B5" s="55" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>BENEDITA</t>
         </is>
@@ -4174,7 +4174,7 @@
       <c r="B6" s="56" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>BORTOLOTI</t>
         </is>
@@ -4182,7 +4182,7 @@
       <c r="B7" s="57" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
@@ -4190,7 +4190,7 @@
       <c r="B8" s="58" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
@@ -4198,7 +4198,7 @@
       <c r="B9" s="59" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>DAVI</t>
         </is>
@@ -4206,7 +4206,7 @@
       <c r="B10" s="60" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>DINO</t>
         </is>
@@ -4214,7 +4214,7 @@
       <c r="B11" s="61" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>DRIELLI</t>
         </is>
@@ -4222,7 +4222,7 @@
       <c r="B12" s="62" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>EUNICE</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="B13" s="63" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>GERALDO</t>
         </is>
@@ -4238,7 +4238,7 @@
       <c r="B14" s="64" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
@@ -4246,7 +4246,7 @@
       <c r="B15" s="65" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
@@ -4254,7 +4254,7 @@
       <c r="B16" s="66" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
         </is>
@@ -4262,7 +4262,7 @@
       <c r="B17" s="67" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>GISELE</t>
         </is>
@@ -4270,7 +4270,7 @@
       <c r="B18" s="68" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
@@ -4278,7 +4278,7 @@
       <c r="B19" s="69" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
@@ -4286,7 +4286,7 @@
       <c r="B20" s="70" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>LILIANE</t>
         </is>
@@ -4294,7 +4294,7 @@
       <c r="B21" s="71" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>M.EDUARDA</t>
         </is>
@@ -4302,7 +4302,7 @@
       <c r="B22" s="72" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>MARCIA</t>
         </is>
@@ -4310,7 +4310,7 @@
       <c r="B23" s="73" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>MARIANA</t>
         </is>
@@ -4318,7 +4318,7 @@
       <c r="B24" s="74" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>MARINA</t>
         </is>
@@ -4326,7 +4326,7 @@
       <c r="B25" s="75" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
@@ -4334,7 +4334,7 @@
       <c r="B26" s="76" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
@@ -4342,7 +4342,7 @@
       <c r="B27" s="77" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>PAPANONI</t>
         </is>
@@ -4350,7 +4350,7 @@
       <c r="B28" s="78" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
@@ -4358,7 +4358,7 @@
       <c r="B29" s="79" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>RAFAEL</t>
         </is>
@@ -4366,7 +4366,7 @@
       <c r="B30" s="80" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>ROBERTA</t>
         </is>
@@ -4374,7 +4374,7 @@
       <c r="B31" s="81" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>ROMARIO</t>
         </is>
@@ -4382,7 +4382,7 @@
       <c r="B32" s="82" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>SAMIA</t>
         </is>
@@ -4390,7 +4390,7 @@
       <c r="B33" s="83" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>SELMA</t>
         </is>
@@ -4398,7 +4398,7 @@
       <c r="B34" s="84" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>SILVANA</t>
         </is>
@@ -4406,7 +4406,7 @@
       <c r="B35" s="85" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t>SILVIA</t>
         </is>
@@ -4414,7 +4414,7 @@
       <c r="B36" s="86" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="0" t="inlineStr">
         <is>
           <t>SIMARA</t>
         </is>
@@ -4422,7 +4422,7 @@
       <c r="B37" s="87" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>THOMAZ</t>
         </is>
@@ -4430,7 +4430,7 @@
       <c r="B38" s="88" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
         <is>
           <t>VINICIUS</t>
         </is>

</xml_diff>

<commit_message>
Remover scripts de otimização obsoletos para agendamento de professores
</commit_message>
<xml_diff>
--- a/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
+++ b/Manha_Ferrucio_2026_SEM_CHOQUES.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="I3" s="18" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="J3" s="20" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="H4" s="23" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="I4" s="26" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="O4" s="29" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>THOMAZ- HIST</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
+          <t>MARINA- REDAÇÃO</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="J5" s="21" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="G9" s="30" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="G10" s="30" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="I10" s="16" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
       <c r="E11" s="31" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
+          <t>SILVANA- RED</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="I11" s="24" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>ALINE- SOC</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1572,12 @@
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
+          <t>SILVANA- RED</t>
         </is>
       </c>
       <c r="H12" s="30" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="I12" s="24" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="O12" s="18" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>ALINE- SOC</t>
         </is>
       </c>
     </row>
@@ -1664,19 +1664,19 @@
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
           <t>MARCIA- ARTE</t>
         </is>
       </c>
-      <c r="H14" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I14" s="30" t="inlineStr">
-        <is>
-          <t>MARINA- REDAÇÃO</t>
-        </is>
-      </c>
       <c r="J14" s="35" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="K14" s="25" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="L14" s="16" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="O14" s="19" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>SILVIA- MAT</t>
+        </is>
+      </c>
+      <c r="I15" s="30" t="inlineStr">
+        <is>
           <t>MARCIA- ARTE</t>
-        </is>
-      </c>
-      <c r="H15" s="24" t="inlineStr">
-        <is>
-          <t>SILVIA- MAT</t>
-        </is>
-      </c>
-      <c r="I15" s="30" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J15" s="25" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -1810,12 +1810,12 @@
       </c>
       <c r="G16" s="22" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="I16" s="17" t="inlineStr">
@@ -1840,17 +1840,17 @@
       </c>
       <c r="M16" s="25" t="inlineStr">
         <is>
+          <t>GERALDO- MAT</t>
+        </is>
+      </c>
+      <c r="N16" s="37" t="inlineStr">
+        <is>
+          <t>SIMARA- OE LP</t>
+        </is>
+      </c>
+      <c r="O16" s="23" t="inlineStr">
+        <is>
           <t>GISELE- ED. FÍSICA</t>
-        </is>
-      </c>
-      <c r="N16" s="37" t="inlineStr">
-        <is>
-          <t>M.EDUARDA- PORT</t>
-        </is>
-      </c>
-      <c r="O16" s="23" t="inlineStr">
-        <is>
-          <t>GERALDO- EMPREEN</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1881,17 +1881,17 @@
       </c>
       <c r="G17" s="22" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>DAVI- FÍSICA</t>
         </is>
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="I17" s="18" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="E18" s="28" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="I18" s="26" t="inlineStr">
         <is>
-          <t>MARINA- REDAÇÃO</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="J18" s="34" t="inlineStr">
@@ -1972,12 +1972,12 @@
       </c>
       <c r="K18" s="38" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="L18" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>DAVI- EFIN</t>
         </is>
       </c>
       <c r="M18" s="29" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="E19" s="28" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
@@ -2038,17 +2038,17 @@
       </c>
       <c r="J19" s="40" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>RAFAEL- ED. FÍSICA</t>
         </is>
       </c>
       <c r="K19" s="38" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="L19" s="22" t="inlineStr">
         <is>
-          <t>DAVI- FÍSICA</t>
+          <t>DAVI- EFIN</t>
         </is>
       </c>
       <c r="M19" s="41" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
+          <t>SILVANA- RED</t>
         </is>
       </c>
       <c r="G21" s="26" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="L21" s="18" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>ALINE- ORATÓRIA</t>
         </is>
       </c>
       <c r="M21" s="41" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="N21" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
       <c r="O21" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>THOMAZ- HIST</t>
         </is>
       </c>
       <c r="D22" s="28" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
-          <t>SILVANA- PORT</t>
+          <t>SILVANA- RED</t>
         </is>
       </c>
       <c r="G22" s="26" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="L22" s="18" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>ALINE- ORATÓRIA</t>
         </is>
       </c>
       <c r="M22" s="41" t="inlineStr">
@@ -2221,12 +2221,12 @@
       </c>
       <c r="N22" s="25" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="O22" s="19" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="H23" s="16" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="I23" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- EFIN</t>
         </is>
       </c>
       <c r="J23" s="17" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="K23" s="25" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="L23" s="34" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="O23" s="26" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -2312,12 +2312,12 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D24" s="30" t="inlineStr">
         <is>
-          <t>DAVI- MAT</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>ALINE- BIO</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I24" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- EFIN</t>
         </is>
       </c>
       <c r="J24" s="34" t="inlineStr">
@@ -2352,12 +2352,12 @@
       </c>
       <c r="K24" s="25" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="L24" s="23" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="M24" s="42" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="O24" s="29" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>M.EDUARDA- PORT</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="D25" s="22" t="inlineStr">
@@ -2418,19 +2418,19 @@
       </c>
       <c r="J25" s="38" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="K25" s="26" t="inlineStr">
         <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="L25" s="18" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="L25" s="18" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
       <c r="M25" s="43" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
@@ -2438,12 +2438,12 @@
       </c>
       <c r="N25" s="37" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>SIMARA- OE LP</t>
         </is>
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>THOMAZ- HIST</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="D26" s="22" t="inlineStr">
@@ -2489,19 +2489,19 @@
       </c>
       <c r="J26" s="38" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>BENEDITA- GEO</t>
         </is>
       </c>
       <c r="K26" s="26" t="inlineStr">
         <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="L26" s="18" t="inlineStr">
+        <is>
           <t>ALINE- BIO</t>
         </is>
       </c>
-      <c r="L26" s="18" t="inlineStr">
-        <is>
-          <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
       <c r="M26" s="44" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
     </row>
@@ -2556,12 +2556,12 @@
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="F28" s="45" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
@@ -2576,12 +2576,12 @@
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
+          <t>ALINE- FILOSOFIA</t>
+        </is>
+      </c>
+      <c r="J28" s="26" t="inlineStr">
+        <is>
           <t>VINICIUS- QUIMICA</t>
-        </is>
-      </c>
-      <c r="J28" s="26" t="inlineStr">
-        <is>
-          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="K28" s="16" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="F29" s="45" t="inlineStr">
         <is>
-          <t>GISELE- ED. FÍSICA</t>
+          <t>PAPANONI- ED. FINAN</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="J29" s="26" t="inlineStr">
         <is>
-          <t>GERALDO- MAT</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="O29" s="49" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>VINICIUS- QUIMICA</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="J30" s="17" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="J31" s="16" t="inlineStr">
@@ -2818,12 +2818,12 @@
       </c>
       <c r="N31" s="25" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>GERALDO- MAT</t>
         </is>
       </c>
       <c r="O31" s="26" t="inlineStr">
         <is>
-          <t>GERALDO- EMPREEN</t>
+          <t>VINICIUS- AP QUIM</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE LP</t>
+          <t>MARINA- PORT</t>
         </is>
       </c>
       <c r="D32" s="48" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>GERALDO- OE MAT</t>
+          <t>ROMARIO- ED FÍSICA</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>ALINE- FILOSOFIA</t>
         </is>
       </c>
       <c r="G32" s="46" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="H32" s="30" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="I32" s="22" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="N32" s="17" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>EUNICE- ATUALID</t>
         </is>
       </c>
       <c r="O32" s="24" t="inlineStr">
@@ -2920,34 +2920,34 @@
       </c>
       <c r="F33" s="26" t="inlineStr">
         <is>
+          <t>VINICIUS- QUIMICA</t>
+        </is>
+      </c>
+      <c r="G33" s="46" t="inlineStr">
+        <is>
+          <t>LILIANE- ED. FINAN</t>
+        </is>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>MARINA- REDAÇÃO</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>EUNICE- HIST</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>ALEXANDRE- ING</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
           <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
-      <c r="G33" s="46" t="inlineStr">
-        <is>
-          <t>LILIANE- ED. FINAN</t>
-        </is>
-      </c>
-      <c r="H33" s="19" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
-      <c r="I33" s="17" t="inlineStr">
-        <is>
-          <t>EUNICE- HIST</t>
-        </is>
-      </c>
-      <c r="J33" s="13" t="inlineStr">
-        <is>
-          <t>ALEXANDRE- ING</t>
-        </is>
-      </c>
-      <c r="K33" s="23" t="inlineStr">
-        <is>
-          <t>ALINE- BIO</t>
-        </is>
-      </c>
       <c r="L33" s="16" t="inlineStr">
         <is>
           <t>SILVANA- PORT</t>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="N33" s="24" t="inlineStr">
         <is>
-          <t>SILVIA- MAT</t>
+          <t>SILVIA- OE MAT</t>
         </is>
       </c>
       <c r="O33" s="34" t="inlineStr">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARINA- REDAÇÃO</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
@@ -3017,12 +3017,12 @@
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="H35" s="26" t="inlineStr">
         <is>
-          <t>ALINE- BIO</t>
+          <t>VINICIUS- QUIMICA</t>
         </is>
       </c>
       <c r="I35" s="24" t="inlineStr">
@@ -3073,12 +3073,12 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>ROMARIO- ED FÍSICA</t>
+          <t>MARINA- OE PORT</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
         <is>
-          <t>MARINA- OE PORT</t>
+          <t>MARCIA- ARTE</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>MARCIA- ARTE</t>
+          <t>GISELE- ED. FÍSICA</t>
         </is>
       </c>
       <c r="H36" s="22" t="inlineStr">
@@ -3123,12 +3123,12 @@
       </c>
       <c r="N36" s="17" t="inlineStr">
         <is>
-          <t>M.EDUARDA- PORT</t>
+          <t>EUNICE- ATUALID</t>
         </is>
       </c>
       <c r="O36" s="49" t="inlineStr">
         <is>
-          <t>EUNICE- HIST</t>
+          <t>BORTOLOTI- PROG</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ALEXANDRE</t>
         </is>
@@ -4142,7 +4142,7 @@
       <c r="B2" s="52" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="0" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ALINE</t>
         </is>
@@ -4150,7 +4150,7 @@
       <c r="B3" s="53" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="0" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>ANDREA</t>
         </is>
@@ -4158,7 +4158,7 @@
       <c r="B4" s="54" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="0" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>BAQUETE</t>
         </is>
@@ -4166,7 +4166,7 @@
       <c r="B5" s="55" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="0" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>BENEDITA</t>
         </is>
@@ -4174,7 +4174,7 @@
       <c r="B6" s="56" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="0" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>BORTOLOTI</t>
         </is>
@@ -4182,7 +4182,7 @@
       <c r="B7" s="57" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="0" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>CARREIRA E COMP</t>
         </is>
@@ -4190,7 +4190,7 @@
       <c r="B8" s="58" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="0" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>COMUNICAÇÃO</t>
         </is>
@@ -4198,7 +4198,7 @@
       <c r="B9" s="59" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="0" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>DAVI</t>
         </is>
@@ -4206,7 +4206,7 @@
       <c r="B10" s="60" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="0" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>DINO</t>
         </is>
@@ -4214,7 +4214,7 @@
       <c r="B11" s="61" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="0" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>DRIELLI</t>
         </is>
@@ -4222,7 +4222,7 @@
       <c r="B12" s="62" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="0" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>EUNICE</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="B13" s="63" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="0" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>GERALDO</t>
         </is>
@@ -4238,7 +4238,7 @@
       <c r="B14" s="64" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="0" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>GEST. FINANCEIRA</t>
         </is>
@@ -4246,7 +4246,7 @@
       <c r="B15" s="65" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="0" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>GESTÃO DE OPERAÇÕES</t>
         </is>
@@ -4254,7 +4254,7 @@
       <c r="B16" s="66" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="0" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>GESTÃO FINANCEIRA</t>
         </is>
@@ -4262,7 +4262,7 @@
       <c r="B17" s="67" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="0" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>GISELE</t>
         </is>
@@ -4270,7 +4270,7 @@
       <c r="B18" s="68" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="0" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>INOVAÇÃO E DES</t>
         </is>
@@ -4278,7 +4278,7 @@
       <c r="B19" s="69" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="0" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>INTRODUÇÃO ADM</t>
         </is>
@@ -4286,7 +4286,7 @@
       <c r="B20" s="70" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="0" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>LILIANE</t>
         </is>
@@ -4294,7 +4294,7 @@
       <c r="B21" s="71" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="0" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>M.EDUARDA</t>
         </is>
@@ -4302,7 +4302,7 @@
       <c r="B22" s="72" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="0" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>MARCIA</t>
         </is>
@@ -4310,7 +4310,7 @@
       <c r="B23" s="73" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="0" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>MARIANA</t>
         </is>
@@ -4318,7 +4318,7 @@
       <c r="B24" s="74" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="0" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>MARINA</t>
         </is>
@@ -4326,7 +4326,7 @@
       <c r="B25" s="75" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="0" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>MARKETING</t>
         </is>
@@ -4334,7 +4334,7 @@
       <c r="B26" s="76" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="0" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>MAT APLICADA</t>
         </is>
@@ -4342,7 +4342,7 @@
       <c r="B27" s="77" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="0" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>PAPANONI</t>
         </is>
@@ -4350,7 +4350,7 @@
       <c r="B28" s="78" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="0" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>PROJETO MULTI</t>
         </is>
@@ -4358,7 +4358,7 @@
       <c r="B29" s="79" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="0" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>RAFAEL</t>
         </is>
@@ -4366,7 +4366,7 @@
       <c r="B30" s="80" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="0" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>ROBERTA</t>
         </is>
@@ -4374,7 +4374,7 @@
       <c r="B31" s="81" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="0" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>ROMARIO</t>
         </is>
@@ -4382,7 +4382,7 @@
       <c r="B32" s="82" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="0" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>SAMIA</t>
         </is>
@@ -4390,7 +4390,7 @@
       <c r="B33" s="83" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="0" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>SELMA</t>
         </is>
@@ -4398,7 +4398,7 @@
       <c r="B34" s="84" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="0" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>SILVANA</t>
         </is>
@@ -4406,7 +4406,7 @@
       <c r="B35" s="85" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="0" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>SILVIA</t>
         </is>
@@ -4414,7 +4414,7 @@
       <c r="B36" s="86" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="0" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>SIMARA</t>
         </is>
@@ -4422,7 +4422,7 @@
       <c r="B37" s="87" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="0" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>THOMAZ</t>
         </is>
@@ -4430,7 +4430,7 @@
       <c r="B38" s="88" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="0" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>VINICIUS</t>
         </is>

</xml_diff>